<commit_message>
feat: update voice bot API implementation, logger, prompting, session manager, and test cases
</commit_message>
<xml_diff>
--- a/test_cases_Excel_byClaude/TestCases_Nhap_3KichBan.xlsx
+++ b/test_cases_Excel_byClaude/TestCases_Nhap_3KichBan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vovinhloc/myworking/customer/cnta/voice_bot/voice_bot/test_cases_Excel_byClaude/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E982EE53-D036-904D-BA90-B2148C7ECA3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89140BB-7A3D-F544-AD9F-69A246181221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -587,7 +587,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -638,6 +638,12 @@
       <sz val="10"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFE0E0E0"/>
+      <name val="Menlo"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -706,7 +712,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -741,26 +747,27 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1071,7 +1078,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -1081,7 +1088,7 @@
       <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -1092,7 +1099,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="12"/>
+      <c r="B4" s="18"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
@@ -1102,7 +1109,7 @@
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="12"/>
+      <c r="B5" s="18"/>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -1112,7 +1119,7 @@
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="13"/>
@@ -1124,7 +1131,7 @@
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="13"/>
@@ -1136,7 +1143,7 @@
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="18" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="13"/>
@@ -1146,7 +1153,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
-      <c r="B9" s="12"/>
+      <c r="B9" s="18"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
@@ -1156,7 +1163,7 @@
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="12"/>
+      <c r="B10" s="18"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
@@ -1166,7 +1173,7 @@
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="18" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="13"/>
@@ -1178,7 +1185,7 @@
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="18" t="s">
         <v>13</v>
       </c>
       <c r="C12" s="13"/>
@@ -1190,7 +1197,7 @@
       <c r="A13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="18" t="s">
         <v>15</v>
       </c>
       <c r="C13" s="13"/>
@@ -1202,7 +1209,7 @@
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="18" t="s">
         <v>17</v>
       </c>
       <c r="C14" s="13"/>
@@ -1212,7 +1219,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="12"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>
@@ -1222,7 +1229,7 @@
       <c r="A16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="18" t="s">
         <v>19</v>
       </c>
       <c r="C16" s="13"/>
@@ -1268,7 +1275,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="13"/>
@@ -1280,7 +1287,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="3" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="17" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="13"/>
@@ -1298,12 +1305,12 @@
       <c r="B4" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
     </row>
     <row r="5" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
@@ -1312,12 +1319,12 @@
       <c r="B5" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
     </row>
     <row r="6" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -1326,12 +1333,12 @@
       <c r="B6" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
     </row>
     <row r="7" spans="1:8" ht="56" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
@@ -1340,12 +1347,12 @@
       <c r="B7" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:8" ht="84" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
@@ -1354,15 +1361,15 @@
       <c r="B8" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
     </row>
     <row r="10" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="13"/>
@@ -1377,15 +1384,15 @@
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
@@ -1394,12 +1401,12 @@
       <c r="B12" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
@@ -1408,12 +1415,12 @@
       <c r="B13" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
@@ -1422,12 +1429,12 @@
       <c r="B14" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
@@ -1436,12 +1443,12 @@
       <c r="B15" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
@@ -1450,12 +1457,12 @@
       <c r="B16" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
@@ -1464,12 +1471,12 @@
       <c r="B17" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
@@ -1478,12 +1485,12 @@
       <c r="B18" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
@@ -1492,15 +1499,15 @@
       <c r="B19" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
     </row>
     <row r="21" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="17" t="s">
         <v>45</v>
       </c>
       <c r="B21" s="13"/>
@@ -1568,7 +1575,9 @@
       <c r="D24" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="11"/>
+      <c r="E24" s="20">
+        <v>15123890724</v>
+      </c>
       <c r="F24" s="11"/>
       <c r="G24" s="11"/>
       <c r="H24" s="11"/>
@@ -1809,24 +1818,24 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B7:H7"/>
     <mergeCell ref="B14:H14"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B18:H18"/>
     <mergeCell ref="B13:H13"/>
     <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B7:H7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1848,7 +1857,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>95</v>
       </c>
       <c r="B1" s="13"/>
@@ -1860,7 +1869,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="3" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="17" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="13"/>
@@ -1878,12 +1887,12 @@
       <c r="B4" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
     </row>
     <row r="5" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
@@ -1892,12 +1901,12 @@
       <c r="B5" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
     </row>
     <row r="6" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -1906,12 +1915,12 @@
       <c r="B6" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
     </row>
     <row r="7" spans="1:8" ht="56" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
@@ -1920,12 +1929,12 @@
       <c r="B7" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:8" ht="84" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
@@ -1934,15 +1943,15 @@
       <c r="B8" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
     </row>
     <row r="10" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="13"/>
@@ -1957,15 +1966,15 @@
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
@@ -1974,12 +1983,12 @@
       <c r="B12" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
@@ -1988,12 +1997,12 @@
       <c r="B13" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
@@ -2002,12 +2011,12 @@
       <c r="B14" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
@@ -2016,12 +2025,12 @@
       <c r="B15" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
@@ -2030,12 +2039,12 @@
       <c r="B16" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
@@ -2044,12 +2053,12 @@
       <c r="B17" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
@@ -2058,12 +2067,12 @@
       <c r="B18" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
@@ -2072,15 +2081,15 @@
       <c r="B19" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
     </row>
     <row r="21" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="17" t="s">
         <v>45</v>
       </c>
       <c r="B21" s="13"/>
@@ -2317,24 +2326,24 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B7:H7"/>
     <mergeCell ref="B14:H14"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B18:H18"/>
     <mergeCell ref="B13:H13"/>
     <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B7:H7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2356,7 +2365,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>141</v>
       </c>
       <c r="B1" s="13"/>
@@ -2368,7 +2377,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="3" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="17" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="13"/>
@@ -2386,12 +2395,12 @@
       <c r="B4" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
     </row>
     <row r="5" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
@@ -2400,12 +2409,12 @@
       <c r="B5" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
     </row>
     <row r="6" spans="1:8" ht="42" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -2414,12 +2423,12 @@
       <c r="B6" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
     </row>
     <row r="7" spans="1:8" ht="56" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
@@ -2428,12 +2437,12 @@
       <c r="B7" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:8" ht="84" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
@@ -2442,15 +2451,15 @@
       <c r="B8" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
     </row>
     <row r="10" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="13"/>
@@ -2465,15 +2474,15 @@
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
@@ -2482,12 +2491,12 @@
       <c r="B12" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
@@ -2496,12 +2505,12 @@
       <c r="B13" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
@@ -2510,12 +2519,12 @@
       <c r="B14" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
@@ -2524,12 +2533,12 @@
       <c r="B15" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
@@ -2538,12 +2547,12 @@
       <c r="B16" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
@@ -2552,12 +2561,12 @@
       <c r="B17" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
@@ -2566,12 +2575,12 @@
       <c r="B18" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
@@ -2580,15 +2589,15 @@
       <c r="B19" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
     </row>
     <row r="21" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="17" t="s">
         <v>45</v>
       </c>
       <c r="B21" s="13"/>
@@ -2843,24 +2852,24 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B7:H7"/>
     <mergeCell ref="B14:H14"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B18:H18"/>
     <mergeCell ref="B13:H13"/>
     <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B7:H7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>